<commit_message>
Update berita 2026-08-11 18:47 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-12.xlsx
+++ b/data/berita_2026-08-12.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -997,8 +997,384 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Dubes Witjaksono tegaskan tekad ASEAN perkuat kemitraan dengan Kenya</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:27:25 +0700</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Duta Besar RI untuk Kenya TBH Witjaksono Adji menegaskan komitmen ASEAN untuk terus memperluas kemitraan di luar ...</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690117/dubes-witjaksono-tegaskan-tekad-asean-perkuat-kemitraan-dengan-kenya</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/WhatsApp-Image-2026-08-11-at-19.08.43.jpeg</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Menhub pastikan seluruh rekomendasi BPK ditindaklanjuti</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:17:22 +0700</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Menteri Perhubungan (Menhub) Dudy Purwagandhi memastikan seluruh rekomendasi Badan Pemeriksa Keuangan (BPK) ...</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690113/menhub-pastikan-seluruh-rekomendasi-bpk-ditindaklanjuti</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/9A3CF4B6-CCC1-4215-AD4D-0C7AA714D87F.jpeg</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Kemensetneg gelar rapat pleno, matangkan rangkaian peringatan HUT RI</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:12:53 +0700</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Kementerian Sekretariat Negara menggelar rapat pleno persiapan rangkaian Bulan Kemerdekaan menjelang peringatan HUT ...</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690111/kemensetneg-gelar-rapat-pleno-matangkan-rangkaian-peringatan-hut-ri</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/1000404279.jpg</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>7 Kantor Pemkab Puncak Papua Tengah Dibakar Massa: Gedung Bupati-DPRD</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:24:48 +0700</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Paulus Pulo</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Massa membakar tujuh kantor pemerintah di Puncak, Papua Tengah, termasuk Kantor Bupati dan DPRD, akibat ketidakpuasan pembagian dana desa.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614538/7-kantor-pemkab-puncak-papua-tengah-dibakar-massa-gedung-bupati-dprd</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/gedung-pemerintahan-di-puncak-papua-tengah-dibakar-massa-1786452308073_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kemenhut Ungkap Jual-Beli Lahan Hutan Lindung di Sulsel, 3 Orang Ditangkap</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:01:12 +0700</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Kemenhut ungkap modus jual-beli lahan hutan lindung di Sulsel. Tiga pelaku ditangkap saat menggarap lahan ilegal.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614536/kemenhut-ungkap-jual-beli-lahan-hutan-lindung-di-sulsel-3-orang-ditangkap</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/12/kemenhut-ungkap-modus-jual-beli-lahan-hutan-lindung-di-sulsel-dok-antara-1786469730093_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Peringatan ke Pegawai, Gus Ipul: Jangan Kebiasaan Habiskan Uang dan Belanja Sembarangan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:47:38 +0700</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Mensos Saifullah Yusuf atau Gus Ipul memperingatkan pegawainya agar meninggalkan kebiasaan menghabiskan uang dan belanja anggaran secara sembarangan.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/11/23324151/peringatan-ke-pegawai-gus-ipul-jangan-kebiasaan-habiskan-uang-dan-belanja</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/pKspNR1Miw68Cgbca6xdXgMI_PM=/425x148:3753x2367/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/05/6a73165e5e027.jpeg</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Perang AS Temui Menhan Sjafrie, Bahas soal Kelanjutan Kerja Sama Pertahanan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:47:38 +0700</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Perang Amerika Serikat (AS) bidang Kebijakan Elbridge A. Colby mengunjungi Menteri Pertahanan RI Sjafrie Sjamsoeddin di Kemenhan RI.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/11/22202711/wakil-menteri-perang-as-temui-menhan-sjafrie-bahas-soal-kelanjutan-kerja</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/d6iy2gqD10-O_Sn9zLIxhlhGQOI=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/11/6a7b340b0529f.jpg</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Rinaldi Umar Batal Dilantik Jadi Dirdik Jampidsus, Ini Alasan Kejagung</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:47:38 +0700</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Alasan Rinaldi Umar batal dilantik sebagai Direktur Penyidikan (Dirdik) pada Jaksa Agung Muda Tindak Pidana Khusus karena alasan pengalaman.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/11/21262681/rinaldi-umar-batal-dilantik-jadi-dirdik-jampidsus-ini-alasan-kejagung</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/RkjlvY0ly1nBMPQx3Rv8uJ7Vyts=/265x66:1297x754/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/03/6a70a42491bfb.jpg</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I12"/>
+  <autoFilter ref="A1:I20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 19:58 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-12.xlsx
+++ b/data/berita_2026-08-12.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1373,8 +1373,337 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mengunjungi Museum Linggam Cahaya, mengulik sejarah mata uang SKR</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:54:39 +0700</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ANTARA - Di sebuah pulau di Kabupaten Lingga, Kepulauan Riau, berdiri sebuah Museum Linggam Cahaya Pulau Daik ...</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5690120/mengunjungi-museum-linggam-cahaya-mengulik-sejarah-mata-uang-skr</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MENGUNJUNGI-MUSEUM-LINGGAM-CAHAYA-MENGULIK-SEJARAH-MATA-UANG-SKR.jpg</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Polisi Kumpulkan Barang Bukti Terkait Kasus Hafalan Qur'an demi Miras</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 02:34:34 +0700</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Polisi selidiki dugaan penistaan agama terkait challenge hafalan Al-Qur'an demi miras di festival musik Ancol. Barang bukti sedang dikumpulkan.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614542/polisi-kumpulkan-barang-bukti-terkait-kasus-hafalan-quran-demi-miras</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/04/09/waduh-di-china-ada-tren-baru-mukbang-minum-miras-yang-berbahaya-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kemlu: 3 ABK WNI Diserang Rudal Houthi di Selat Bab Al-Mandeb</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 02:02:55 +0700</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Kemlu RI mengonfirmasi serangan Houthi di Selat Al-Mandeb yang melibatkan tiga ABK WNI. Dua dilaporkan terluka dan satu dilaporkan tewas masih dikonfirmasi.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614540/kemlu-3-abk-wni-diserang-rudal-houthi-di-selat-bab-al-mandeb</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/30/direktur-perlindungan-wni-kementerian-luar-negeri-kemlu-heni-hamidah-1777527020619_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Berapa Kali Sebaiknya Medical Check Up dalam Setahun? Ini Penjelasan Dokter</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 02:30:20 +0700</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Menurut Dokter Spesialis Patologi Klinik RS PKU Muhammadiyah Surakarta, dr. Hapsary Puteri,  seseorang disarankan melakukan MCU setahun sekali.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7867147/berapa-kali-sebaiknya-medical-check-up-dalam-setahun-ini-penjelasan-dokter</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/h9Iwq3jQiUY5KGuceYOueGo4SFg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-medical-check-up-istimewa-jk.jpg</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>5 Tempat Persembunyian Donald Trump: Terbaru di Dalam Truk Katering</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 02:02:21 +0700</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Trump beberapa kali harus disembunyikan demi keamanan, termasuk saat dipindahkan dengan truk katering bandara karena ancaman Iran</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867146/5-tempat-persembunyian-donald-trump-terbaru-di-dalam-truk-katering</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/G_fSln9DwkqFdZKehzhyGyDgAgw=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Donald-T1rump-melakukan-konferensi-si.jpg</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1 Juta Sarjana Menganggur, Pakar Soroti Ketidakseimbangan Jumlah Lulusan dan Daya Serap Pasar Kerja</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:20:16 +0700</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Menurut data pada Mei 2026, jumlah penduduk yang tidak bekerja sebanyak 7,22 juta orang, sekitar 14,31 persen di antaranya adalah lulusan sarjana.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867145/1-juta-sarjana-menganggur-pakar-soroti-ketidakseimbangan-jumlah-lulusan-dan-daya-serap-pasar-kerja</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/DPX12N-mX0CtRVfqOLpyiUHnrwE=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-peraih-gelar-sarjana-9.jpg</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sistem Air di 12 Negara Bagian AS Diretas, Iran Dicurigai sebagai Dalang</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 01:03:29 +0700</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Serangan siber menyasar sistem air di sedikitnya tujuh negara bagian AS, termasuk lebih dari 30 sistem di Minnesota.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867144/sistem-air-di-12-negara-bagian-as-diretas-iran-dicurigai-sebagai-dalang</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/-iLI2GIlawBLJIXGkQMMdQkM2aA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Tangkap-layar-YouTube-ABC-News-memperlihatkan-contoh-sistem-air-di-Am.jpg</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I20"/>
+  <autoFilter ref="A1:I27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 20:35 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-12.xlsx
+++ b/data/berita_2026-08-12.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -1702,8 +1702,102 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Pabrik Bingkai di Duren Sawit Jaktim Kebakaran, 22 Unit Damkar Dikerahkan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 03:07:06 +0700</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Azhar Bagas Ramadhan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Kebakaran melanda pabrik bingkai di Duren Sawit, Jakarta Timur. 100 personel damkar dikerahkan, namun terkendala akses dan sumber air. Penyebab belum diketahui.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614543/pabrik-bingkai-di-duren-sawit-jaktim-kebakaran-22-unit-damkar-dikerahkan</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/12/kebakaran-pabrik-bingkai-di-duren-sawit-jaktim-rabu-128-dini-hari-dok-istimewa-1786478796541_34.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Profil Nasaruddin Umar, Menteri Agama yang Berpeluang Jadi Calon Ketua Umum PBNU</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 03:02:11 +0700</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Menteri Agama K.H. Nasaruddin Umar disebut berpeluang maju menjadi calon Ketua Umum Pengurus Besar Nahdlatul Ulama (PBNU).</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867148/profil-nasaruddin-umar-menteri-agama-yang-berpeluang-jadi-calon-ketua-umum-pbnu</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ZHG5-J1vu7NxJTscg7aMzkVoL3o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Menteri-Agama-Nasaruddin-Umar-1111.jpg</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I27"/>
+  <autoFilter ref="A1:I29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 21:38 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-12.xlsx
+++ b/data/berita_2026-08-12.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1796,8 +1796,666 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Emery nilai melawan PSG  ujian bagus</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:14:16 +0700</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Pelatih Aston Villa Unai Emery menilai laga melawan Paris Saint-Germain (PSG) dalam  Piala Super Eropa di Stadion ...</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690147/emery-nilai-melawan-psg-ujian-bagus</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/image-41.jpg</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PSG antusias sambut laga Piala Super lawan Aston Villa</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:08:18 +0700</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Pelatih Paris Saint-Germain (PSG) Luis Enrique mengatakan timnya antusiastis  menyambut laga Piala Super Eropa ...</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690145/psg-antusias-sambut-laga-piala-super-lawan-aston-villa</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/1U6A2198_fgqcuq.jpg</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>DHL perkuat kesiapan kerja generasi muda lewat GoTeach dan UPGRADE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:04:36 +0700</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>DHL Group memperkuat kesiapan kerja generasi muda Indonesia melalui program GoTeach dan UPGRADE dengan menghadirkan ...</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690143/dhl-perkuat-kesiapan-kerja-generasi-muda-lewat-goteach-dan-upgrade</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/F9894DC9-42C3-46AD-BD3C-4AE394FBF07E.jpeg</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Al Ittihad dan Pakhtakor melangkah ke fase liga ACL Elite</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:02:03 +0700</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Al Ittihad dan Pakthtakor melangkah ke fase liga AFC Champions League (ACL) Elite wilayah barat setelah menyingkirkan ...</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690139/al-ittihad-dan-pakhtakor-melangkah-ke-fase-liga-acl-elite</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/image-40.jpg</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BMKG prakirakan sebagian besar Jakarta cerah di Rabu pagi</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:01:38 +0700</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) memprakirakan sebagian besar wilayah DKI Jakarta dalam kondisi ...</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690136/bmkg-prakirakan-sebagian-besar-jakarta-cerah-di-rabu-pagi</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/19/IMG_20260719_000858.jpg</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Pengamat nilai insentif diperlukan untuk wujudkan zero ODOL di 2027</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 03:57:59 +0700</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Pengamat transportasi dari Inisiasi Strategis Transportasi (Instran) Deddy Herlambang menilai insentif diperlukan untuk ...</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690135/pengamat-nilai-insentif-diperlukan-untuk-wujudkan-zero-odol-di-2027</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/E2F5FB05-5F99-4113-A031-16C9D172E36C.jpeg</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Bardghji terancam absen bela Barcelona karena operasi ligamen</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 03:55:44 +0700</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Gelandang Barcelona Roony Bardghji terancam absen membela Blaugrana karena harus menjalani operasi ligamen pada lutut ...</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690131/bardghji-terancam-absen-bela-barcelona-karena-operasi-ligamen</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/05/16/FCB.jpg</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Pelindo Multi Terminal: Arus barang capai 59,59 juta ton di semester I</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 03:54:24 +0700</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>PT Pelindo Multi Terminal, anak usaha PT Pelabuhan Indonesia (Persero), mencatat arus barang mencapai 59,59 juta ton ...</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690127/pelindo-multi-terminal-arus-barang-capai-5959-juta-ton-di-semester-i</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/897B7F64-B5C0-43BC-9080-8B0E7FEFDA55.jpeg</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Bayi Dikubur di Rumah Pasutri Mojokerto Ternyata Korban Pembunuhan</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:14:29 +0700</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Enggran Eko Budianto</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Kuburan bayi ditemukan di rumah pasutri Mojokerto. Autopsi mengungkap bayi dibunuh setelah lahir, meninggal karena dibekap. Investigasi masih berlanjut.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614548/bayi-dikubur-di-rumah-pasutri-mojokerto-ternyata-korban-pembunuhan</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/pemakaman-bayi-yang-sempat-dikubur-di-rumah-warga-mojokerto-1786443183049_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Hanura Usul Sistem Pemilu 2029 Gabungkan Proporsional Terbuka-Tertutup</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 03:41:06 +0700</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Alamudin Hamapu</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Partai Hanura usulkan sistem pemilu 2029 gabungkan proporsional terbuka dan tertutup. Tujuannya, tingkatkan kualitas anggota DPR dan DPRD.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614546/hanura-usul-sistem-pemilu-2029-gabungkan-proporsional-terbuka-tertutup</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/10/ketua-tim-task-force-hanura-patrice-rio-cappella-di-medan-nizar-aldidetiksumut-1786378134569_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Banyumas, Rabu 12 Agustus 2026: Mayoritas Daerah Cerah</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:12:22 +0700</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Pada hari Rabu, 12 Agustus 2026, sebagian besar daerah Kabupaten Banyumas, Jawa Tengah, akan cerah.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867151/prakiraan-cuaca-banyumas-rabu-12-agustus-2026-mayoritas-daerah-cerah</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/AX_5QI3DZO6kl9mzAYeoSUl6g3A=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Foto-ilustrasi-cuaca-cerah-berawan-ilustrasi-cerah-berawan.jpg</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20 Link Twibbon Hari Gajah Sedunia 2026, Lengkap dengan Cara Mudah Unggah di Media Sosial</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:06:56 +0700</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Link Twibbon Hari Gajah Sedunia 2026, bingkai foto cocok dipakai sebagai foto profil dan diunggah di sosial media pada tanggal 12 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867150/20-link-twibbon-hari-gajah-sedunia-2026-lengkap-dengan-cara-mudah-unggah-di-media-sosial</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PrguIH4HcnLzDzgSnyAolmMdrJU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Link-Twibbon-Hari-Gajah-Sedunia-2026-bingkai-foto.jpg</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Pertumbuhan Ekonomi RI 5,29 Persen, Ferry Latuhihin: Tinggi, tapi Gagal Ciptakan Lapangan Kerja</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 03:33:38 +0700</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Ferry Latuhihin menyebut di Indonesia terjadi immiserizing growth atau pertumbuhan yang justru memiskinkan rakyat.</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867149/pertumbuhan-ekonomi-ri-529-persen-ferry-latuhihin-tinggi-tapi-gagal-ciptakan-lapangan-kerja</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/y096sh1ukVa6j3okWpbaC5lOJ1c=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Konferensi-pers-Badan-Pusat-Statistik-mengenai-pertumbuhan-ekonomi.jpg</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Cuaca Jakarta Rabu Diprediksi Cerah, Suhu Capai 35 Derajat</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:28:13 +0700</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BMKG memprakirakan cuaca Jakarta didominasi cerah dan cerah berawan sepanjang Rabu dengan suhu mencapai 35 derajat Celsius.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267588/cuaca-jakarta-rabu-diprediksi-cerah-suhu-capai-35-derajat</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/3-F2plV7Pg7xWbP2yDN5g6R05rM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/3453943/original/049969200_1620650232-Jakarta_Cerah.jpg</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I29"/>
+  <autoFilter ref="A1:I43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 22:34 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-12.xlsx
+++ b/data/berita_2026-08-12.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,18 +419,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2454,8 +2454,572 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Empat kementerian/lembaga sepakat satu data tangani korban Napza</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:15:40 +0700</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ANTARA - Kementerian Sosial, Kementerian Kesehatan, Kementerian Ketenagakerjaan, dan Badan Narkotika Nasional ...</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5690124/empat-kementerian-lembaga-sepakat-satu-data-tangani-korban-napza</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/EMPAT-KEMENTERIANLEMBAGA-SEPAKAT-SATU-DATA-TANGANI-KORBAN-NAPZA.jpg</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Konser Kemerdekaan GBN 2026 digelar perdana di Bogor</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:09:38 +0700</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ANTARA - Konser Kemerdekaan Gita Bahana Nusantara (GBN) 2026 digelar untuk pertama kalinya di Kabupaten Bogor, tepatnya ...</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5690121/konser-kemerdekaan-gbn-2026-digelar-perdana-di-bogor</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KONSER-KEMERDEKAAN-GBN-2026-DIGELAR-PERDANA-DI-BOGOR.jpg</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Ekshumasi Jasad Sutrismo Digelar Hari Ini, Keluarga Tak Hadir</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:08:36 +0700</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Anang Firmansyah</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Ekshumasi jenazah Sutrimo di Banyumas digelar hari ini tanpa kehadiran keluarga. Kuasa hukum memastikan keluarga siap dan menyerahkan proses kepada hukum.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614557/ekshumasi-jasad-sutrismo-digelar-hari-ini-keluarga-tak-hadir</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/suasana-makam-sutrimo-jelang-ekshumasi-di-desa-wlahar-kecamatan-wangon-kabupaten-banyumas-selasa-1182026-1786435403861_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Nabilah Rahman Dozan Jadi Ibu, Perlihatkan Momen Melahirkan</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:05:45 +0700</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Mauludi Rismoyo</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Ada kabar bahagia dari kreator Nabilah Rahman Dozan. Anak Betharia Sonata-Willy Dozan itu telah menjadi ibu.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8614365/nabilah-rahman-dozan-jadi-ibu-perlihatkan-momen-melahirkan</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/nabilah-rahman-dozan-1786456492508_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>FOTO: Topan Dolphin Bikin Shanghai Kebanjiran</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Topan Dolphin membanjiri sejumlah kawasan di Shanghai, China, pada Senin (10/8).</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260810162823-115-1390688/foto-topan-dolphin-bikin-shanghai-kebanjiran</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/10/topan-dolphin-bikin-shanghai-kebanjiran-1786354080836_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Evakuasi Longsor Imbas Hujan Deras di Baguio Filipina, 10 Orang Tewas</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 03:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Sebanyak 10 orang tewas akibat tanah longsor yang dipicu hujan deras dan banjir di kota Baguio, Filipina utara.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260811143515-110-1391034/evakuasi-longsor-imbas-hujan-deras-di-baguio-filipina-10-orang-tewas</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/11/thumbnail-video-1786433847390_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Respons Lisa Mariana saat Namanya Kembali Dikaitkan dalam Kasus Ridwan Kamil</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:04:08 +0700</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Selebgram Lisa Mariana memberikan respons saat namanya kembali dikaitkan dalam kasus Ridwan Kamil.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7867152/respons-lisa-mariana-saat-namanya-kembali-dikaitkan-dalam-kasus-ridwan-kamil</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/s1l79hkTpSazeGfRNRx-CThSk6w=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Lisa-Mariana-Jalani-Pemeriksaan-Sebagai-Tersangka_20251025_072830.jpg</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>New Xforce HEV, Strategi Mitsubishi Hadirkan Hybrid Sebagai Pilihan yang Lebih Irit</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- Bagi sebagian orang, daya tarik sebuah mobil bukan sekadar tampilan atau banyaknya fitur. Seberapa sering harus berhenti di SPBU, berapa besar biaya yang perlu disiapkan setiap bulan,...</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjm90z348/new-xforce-hev-strategi-mitsubishi-hadirkan-hybrid-sebagai-pilihan-yang-lebih-irit</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/037938500-1785556282-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Kebakaran di Bromo Belum Padam, 2 Titik Api Tersisa di Tebing Curam</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:21:30 +0700</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>​ BNPB Targetkan Karhutlah di Gunung Bromo pad Total Akhir Pekan ini</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267597/kebakaran-di-bromo-belum-padam-2-titik-api-tersisa-di-tebing-curam</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/voWV0fDTfAVK22PREFRzLVP6ees=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321678/original/005690100_1786486848-IMG-20260809-WA0038_copy_1024x683_1.jpg</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Cerita Pilu dari Atas Jalur Kereta Jurangmangu</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:11:39 +0700</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Kasus siswi tertemper kereta di Stasiun Jurangmangu masih menjadi misteri.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267576/cerita-pilu-dari-atas-jalur-kereta-jurangmangu</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/wsCOKo7lwpcHFOmpQEe6udxnRi4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9320985/original/089880800_1786422102-318f8b17-947b-4bbd-b67a-057361f46779.jpg</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Situs Sejarah Bogor Naik Status Cagar Budaya Nasional, Ini Daftarnya</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:41:31 +0700</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Kemenbud menyiapkan sejumlah situs bersejarah di Kabupaten Bogor untuk direvitalisasi dan ditingkatkan statusnya menjadi Cagar Budaya Nasional.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267590/situs-sejarah-bogor-naik-status-cagar-budaya-nasional-ini-daftarnya</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/XKMPbLLXaZ_sGEi7RpoTddXobWU=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321673/original/004543500_1786484142-1003331109.jpg</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Jaksa Beberkan 27 Nama Penerima Uang dari Kasus Korupsi Kuota Haji Khusus</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:43:18 +0700</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Angka yang mengalir ribuan hingga hingga jutaan dolar Amerika Serikat.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267091/jaksa-beberkan-27-nama-penerima-uang-dari-kasus-korupsi-kuota-haji-khusus</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/Kcc9tinbWO-BlcvrzhwjP66t9xo=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321231/original/009653200_1786434165-IMG_20260811_135837_642.jpg</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I43"/>
+  <autoFilter ref="A1:I55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-11 23:32 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-12.xlsx
+++ b/data/berita_2026-08-12.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3018,8 +3018,1230 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>BNN usulkan tim terpadu awasi tempat rehabilitasi narkotika</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:26:42 +0700</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Badan Narkotika Nasional (BNN) mengusulkan pembentukan tim terpadu lintas instansi untuk memperkuat pengawasan terhadap ...</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690156/bnn-usulkan-tim-terpadu-awasi-tempat-rehabilitasi-narkotika</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/1003331133.jpg</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Gedung Biro Kesra Setda Kantor Gubernur Kalteng terbakar</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:17:10 +0700</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Gedung yang digunakan sebagai Biro Kesejahteraan Rakyat (Kesra) Sekretariat Daerah (Setda) Provinsi Kalimantan Tengah ...</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690153/gedung-biro-kesra-setda-kantor-gubernur-kalteng-terbakar</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/1001742010.jpg</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>JPU: Pengaturan kuota haji tambahan "satu pintu" lewat Fuad Hasan</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:05:05 +0700</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Jaksa Penuntut Umum (JPU) dari Komisi Pemberantasan Korupsi (KPK) Fahmi Idris menyebut pengaturan pengisian kuota haji ...</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690151/jpu-pengaturan-kuota-haji-tambahan-satu-pintu-lewat-fuad-hasan</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/18/KPK-periksa-Fuad-Hasan-Masyhur-terkait-korupsi-penyelenggaraan-haji-180626-sth-01A.jpg</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Siaga jaga keamanan acara HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Pengamanan intensif disiapkan guna memastikan seluruh rangkaian acara HUT ke-81 RI di Jakarta berjalan lancar. ...</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5689489/siaga-jaga-keamanan-acara-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/11/20260811-Siaga-jaga-keamanan-acara-HUT-ke-81-RI.jpg</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Deras Kecaman Challenge Hafal Al-Qur'an Berhadiah Miras</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:04:39 +0700</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Aksi tantangan promosi miras berkedok tantangan hafalan Al-Qur'an viral di media sosial. Tindakan itu mendapatkan respons keras berbagai kalangan masyarakat</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614571/deras-kecaman-challenge-hafal-al-quran-berhadiah-miras</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/1144667396-1786419072166_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Pendaftaran Magang Nasional Batch 2 Dibuka Bulan Depan</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:55:44 +0700</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Program magang nasional batch 2 tahun 2026 akan dibuka pertengahan September atau bulan depan.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8613927/pendaftaran-magang-nasional-batch-2-dibuka-bulan-depan</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/06/14/gedung-kemnaker_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Lucky Girl! Potret Gempita Nora Marten Jadi Player Escort AC Milan</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:03:40 +0700</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Gading Marten baru mengunggah momen Gempita menjadi player escort AC Milan dalam laga lawan Chelsea di GBK. Wah... kesempatan yang langka banget ya Gem!</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8614564/lucky-girl-potret-gempita-nora-marten-jadi-player-escort-ac-milan</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/12/gempita-nora-marten-1786473042713_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>BWF Soroti 5 Ganda Putri Kandidat Juara di Kejuaraan Dunia BWF 2026, China Masih Dominan</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:10:45 +0700</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>BWF menyoroti lima pasangan ganda putri yang berpeluang kuat memperebutkan gelar juara Kejuaraan Dunia BWF 2026 di New Delhi.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7867166/bwf-soroti-5-ganda-putri-kandidat-juara-di-kejuaraan-dunia-bwf-2026-china-masih-dominan</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/FVpXNnAKNHPDJwLvMjAxW68URys=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/pasangan-baek-ha-na-dan-lee-so-he-juara-ganda-putri-indonesia-open-2024_20240609_162819.jpg</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Waspada Dokter AI di YouTube dan TikTok, Lansia Jadi Target karena Mudah Percaya Klaim Sembuh Instan</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:05:05 +0700</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Fenomena "dokter AI" kini menjadi perhatian karena kecerdasan buatan dapat dimanfaatkan untuk membuat akun yang tampak seperti akun dokter.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7867165/waspada-dokter-ai-di-youtube-dan-tiktok-lansia-jadi-target-karena-mudah-percaya-klaim-sembuh-instan</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/B2znGZiLatFc4eBlvPbS53WlfhY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-dokter-675755.jpg</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Sengketa Upah Berlanjut, Pekerja Hyundai Motor Akan Mogok Kerja Parsial 4 hari</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:01:27 +0700</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Serikat pekerja Hyundai Motor akan menggelar aksi mogok kerja parsial 4 hari minggu ini setelah gagal mencapai kesepakatan soal upah dengan manajemen.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/otomotif/7867164/sengketa-upah-berlanjutpekerja-hyundai-motor-akan-mogok-kerja-parsial-4-hari</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/wq63QilbG0SiqNAeGylSS7wVfxo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Preskon-Serikat-Pekerja-Hyundai.jpg</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Senpi Dipakai Mantan Istri hingga Tewas, Brigadir Imansyah Dipatsus</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:58:05 +0700</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Iman bukan ditahan karena tindak pidana pembunuhan mantan istri, melainkan dugaan kelalaian senjata apinya digunakan Winda untuk dugaan bunuh diri.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867163/senpi-dipakai-mantan-istri-hingga-tewas-brigadir-imansyah-dipatsus</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tCmUGnrMn3EXKOVRe3-h9sRQHRI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Winda-Lorenza-Gowasa-ditemukan-meninggal.jpg</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Hasil 10 Laga Awal Man City Masih Misteri, Pep Guardiola Bikin Enzo Maresca Sadar Posisi</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:57:56 +0700</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Enzo Maresca sadar bayang-bayang Pep Guardiola akan selalu mengikutinya di Manchester City. Namun, dia merasa terhormat.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867162/hasil-10-laga-awal-man-city-masih-misteri-pep-guardiola-bikin-enzo-maresca-sadar-posisi</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/vfDR7WH13Yq2TymeJufIk9xRI6o=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Enzo-Maresca-Chelsea-412.jpg</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Challenge Hafalan Surat Ad-Dhuha Berhadiah Miras Viral, Ahli Hukum: Polisi Bisa Langsung Bertindak</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:46:34 +0700</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Dugaan penistaan agama melalui challenge hafalan Surat Ad-Dhuha dengan imbalan minuman keras (miras) di sebuah festival musik menjadi sorotan.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7867161/challenge-hafalan-surat-ad-dhuha-berhadiah-miras-viral-ahli-hukum-polisi-bisa-langsung-bertindak</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/uZeNIDQRbmXfRPd3jGtgCkapzCg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Abdul-Fickar-Hadjar-Pakar-Hukum-Pidana-1.jpg</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Terjemahan Lirik Lagu She's The One - Robbie Williams: I was Her, She was Me, We were One</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:43:50 +0700</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Simak terjemahan lirik lagu "She's The One" yang pernah dibawakan oleh penyanyi sekaligus penulis lagu asal Inggris, Robbie Williams.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/musik/7867160/terjemahan-lirik-lagu-shes-the-one-robbie-williams-i-was-her-she-was-me-we-were-one</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/dizVB9x6SK7BSsXjPU6kpy9COv4=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/headset-vd-pink.jpg</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>5 Populer Internasional: Gempa M7,4 di Kolombia - Festival Indonesia di Jepang Berakhir Ricuh</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:43:15 +0700</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Gempa magnitudo 7,4 mengguncang Kolombia, menewaskan 110 orang, melukai puluhan, dan lebih dari 1.400 laporan orang hilang masuk.</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867159/5-populer-internasional-gempa-m74-di-kolombia-festival-indonesia-di-jepang-berakhir-ricuh</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/hzWx5otJiYfuvi7E1WBaYnCcYqs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/KONDISI-KOTA-PEREIRA-SETELAH-GEMPA-GUNCANG-KOLOMBIA.jpg</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Sosok Rico Roberto Syah, Pemuda Beri Mahar Eskavator ke Istri saat Nikah, Anak Kades di Grobogan</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:39:23 +0700</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Rico viral usai memberi mahar ekskavator dan mobil mewah senilai miliaran rupiah, ternyata anak kepala desa dan pengusaha alat berat.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867158/sosok-rico-roberto-syah-pemuda-beri-mahar-eskavator-ke-istri-saat-nikah-anak-kades-di-grobogan</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Lk5EsQgM-2vRsI5Pcqs_dGtaHEY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/P-Sosok-Rico-Roberto-Syah-Pemuda-Beri-Mahar-Eskavator-ke-Istri-saat-Nikah-Anak-Kades-di-Grobogan.jpg</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Wardatina Mawa Ungkap Cara Co-parenting Bersama Insanul Fahmi setelah Resmi Cerai</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:36:38 +0700</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Meski telah resmi berpisah, konten kreator Wardatina Mawa tetap jalani co-parenting bersama Insanul Fahmi.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7867157/wardatina-mawa-ungkap-cara-co-parenting-bersama-insanul-fahmi-setelah-resmi-cerai</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ErCYTFkO3XgNmOrc7eBO-8wiYgM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Wardatina-Mawa-menunjukkan-tanda-bukti-laporan-kepolisian-perselingkuhan-Inara-Rusli.jpg</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Hasil Kualifikasi Liga Champions Tadi Malam: Eks Klub Calvin Verdonk Menang, Penakluk Inter Menggila</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:25:31 +0700</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Drama Kualifikasi Liga Champions 2026/2027! Eks klub Calvin Verdonk, NEC Nijmegen, sukses menyingkirkan Olympiakos, dan kini menuju rekor bersejarah.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867156/hasil-kualifikasi-liga-champions-tadi-malam-eks-klub-calvin-verdonk-menang-penakluk-inter-menggila</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/u5hoK4C9GH03Myg2wW1vEVD9QQs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/gambar-ini-menunjukkan-trofi-liga-champions-uefa-sebelum-pengundian.jpg</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Sulawesi Barat Rabu, 12 Agustus 2026: Mamuju Cerah</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:23:46 +0700</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>BMKG melaporkan prakiraan cuaca untuk wilayah Sulawesi Barat (Sulbar), Rabu (12/8/2026). Mamuju akan cerah hari ini.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867155/prakiraan-cuaca-sulawesi-barat-rabu-12-agustus-2026-mamuju-cerah</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/b6l4ZqXyMCa4bjxdlZtvFOJ6Lbs=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Prakiraan-Cuaca-Sulawesi-Barat.jpg</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>5 Populer Regional: Sosok PPPK Live Medsos saat Jam Kerja - KH Anwar Zahid Alami Kecelakaan</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:22:20 +0700</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>PPPK Bandung Barat viral bahas dugaan fee proyek 1 persen saat jam kerja, sementara mobil KH Anwar Zahid ditabrak truk di Bojonegoro.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867154/5-populer-regional-sosok-pppk-live-medsos-saat-jam-kerja-kh-anwar-zahid-alami-kecelakaan</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Pb-TMS02knqut0jv5amkSddVkvU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Indah-Live-TikTok.jpg</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Trump Diam-diam Dipindah dari Air Force One Pakai Truk Katering demi Hindari Ancaman Iran</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:18:04 +0700</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Trump diam-diam dipindahkan dari Air Force One lewat truk katering ke jet militer setelah muncul ancaman pembunuhan dari Iran.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867153/trump-diam-diam-dipindah-dari-air-force-one-pakai-truk-katering-demi-hindari-ancaman-iran</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Ft6MFHVX9_dtn4yZZXYEToZRi-Y=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/AIR-FORCE-ONE-Tangkap-layar-YouTube-Associated-Press-2-J.jpg</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Mahasiswa Riset SPPG, Dampak ke UMKM dan Ekonomi Lokal Dikaji</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA – Pelaksanaan Satuan Pelayanan Pemenuhan Gizi (SPPG) tidak hanya berkaitan dengan pemenuhan gizi penerima manfaat, tetapi juga memiliki dampak terhadap aktivitas ekonomi di sekitar dapur. Penyerapan UMKM sebagai...</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjm29u416/mahasiswa-riset-sppg-dampak-ke-umkm-dan-ekonomi-lokal-dikaji</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/047822600-1775755284-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Otomotif</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>New Xforce HEV, Strategi Mitsubishi Hadirkan Hybrid Sebagai Pilihan yang Lebih Ekonomis</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 04:50:00 +0700</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Israr Itah</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, TANGERANG -- Bagi sebagian orang, daya tarik sebuah mobil bukan sekadar tampilan atau banyaknya fitur. Seberapa sering harus berhenti di SPBU, berapa besar biaya yang perlu disiapkan setiap bulan,...</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjm90z348/new-xforce-hev-strategi-mitsubishi-hadirkan-hybrid-sebagai-pilihan-yang-lebih-ekonomis</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/037938500-1785556282-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Seleksi Hakim Agung, KY Ungkap Hal yang Bikin Identitas Calon Tersembunyi</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:16:20 +0700</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>KY memastikan seleksi calon hakim agung dan hakim ad hoc 2026 berlangsung transparan dengan melibatkan publik dan menerapkan mekanisme blind review.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267613/seleksi-hakim-agung-ky-ungkap-hal-yang-bikin-identitas-calon-tersembunyi</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/SOZ0nfn8RgmbOySv6A3U2HW6IiM=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/1102777/original/054688000_1452067414-20160106--Ilustrasi-Gedung-Komisi-Yudisial-Hel2.jpg</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Ketika Agama Dibuat Challenge Berhadiah Miras, Tak Ada Alasan Ampuni Pelaku</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Sebuah tantangan di tengah riuh festival musik The Sounds Project di kawasan Ancol mendadak berubah menjadi polemik.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267575/ketika-agama-dibuat-challenge-berhadiah-miras-tak-ada-alasan-ampuni-pelaku</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Fp5iC-vppn7dJSzwqGEBlrLz0gY=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321055/original/059736500_1786425649-Jepretan_Layar_2025-08-11_pukul_12.15.34.jpg</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Pesan Megawati untuk Pimpinan Organisasi Sayap Partai</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:53:56 +0700</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Megawati Soekarnoputri melantik pimpinan organisasi sayap PDIP, meminta kader dekat dengan rakyat. Ia juga menyoroti masalah sarjana menganggur dan menugaskan badan riset mencari solusi.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267610/pesan-megawati-untuk-pimpinan-organisasi-sayap-partai</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/m48HfJYPaJEZKeA4JZOFEYcJ3b0=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321561/original/095047900_1786449805-DSC02530.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I55"/>
+  <autoFilter ref="A1:I81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-12 00:59 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-12.xlsx
+++ b/data/berita_2026-08-12.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -4240,8 +4240,2453 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Rabu, BMKG: Mayoritas kota besar alami berawan-hujan ringan</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:17:53 +0700</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mengeluarkan peringatan dini berupa potensi hujan ringan, sedang ...</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690181/rabu-bmkg-mayoritas-kota-besar-alami-berawan-hujan-ringan</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/08/304062.jpg</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>DKI beri sanksi Rp10 juta kepada penyedia jasa angkut sampah nakal</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:08:50 +0700</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta memberikan sanksi administratif Rp10 juta serta teguran tertulis pertama ...</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690172/dki-beri-sanksi-rp10-juta-kepada-penyedia-jasa-angkut-sampah-nakal</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/1000319700.jpg</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Kemnaker siapkan akses pelatihan-peluang kerja bagi penyintas narkoba</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:57:49 +0700</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Kementerian Ketenagakerjaan (Kemnaker) menyiapkan akses pelatihan dan peluang atau kesempatan kerja bagi penyintas ...</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690168/kemnaker-siapkan-akses-pelatihan-peluang-kerja-bagi-penyintas-narkoba</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/IMG_0820.jpeg</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Gedung Biro Kesra Setda Provinsi Kalteng terbakar</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:17:10 +0700</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Gedung yang digunakan sebagai Biro Kesejahteraan Rakyat (Kesra) Sekretariat Daerah (Setda) Provinsi Kalimantan Tengah ...</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690153/gedung-biro-kesra-setda-provinsi-kalteng-terbakar</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/12/1001742010.jpg</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Cara klaim asuransi mobil: Syarat, dokumen, dan prosedurnya</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:53:35 +0700</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Mengajukan klaim asuransi mobil membutuhkan kelengkapan dokumen dan ketepatan mengikuti prosedur yang ditetapkan ...</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5690216/cara-klaim-asuransi-mobil-syarat-dokumen-dan-prosedurnya</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2017/02/20170201antarafoto-asuransi-astra-310117-ho.jpg</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Ekonomi</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Biaya klaim asuransi mobil berapa? Ini rincian dan contohnya</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:50:53 +0700</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Biaya klaim asuransi mobil tidak selalu sepenuhnya ditanggung perusahaan asuransi. Pemilik kendaraan umumnya tetap ...</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5690211/biaya-klaim-asuransi-mobil-berapa-ini-rincian-dan-contohnya</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/02/03/IMG-20220203-WA0036.jpg</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Politik</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Paskibra vs Paskibraka: Ini perbedaan dan tugasnya</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:41:01 +0700</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Paskibra dan Paskibraka sama-sama berkaitan dengan tugas pengibaran bendera Merah Putih. Namun, keduanya memiliki ...</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690197/paskibra-vs-paskibraka-ini-perbedaan-dan-tugasnya</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/09/latihan-paskibraka-di-sulawesi-barat-2837643.jpg</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Politik</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Formasi 17-8-45 Paskibraka: Sejarah dan makna di baliknya</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:37:14 +0700</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Formasi 17-8-45 menjadi bagian penting dalam pelaksanaan tugas Pasukan Pengibar Bendera Pusaka (Paskibraka) pada ...</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5690195/formasi-17-8-45-paskibraka-sejarah-dan-makna-di-baliknya</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/10/1003327208.jpg</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Karhutla Belum Padam, Penutupan Bromo Diperpanjang hingga 15 Agustus</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:29:36 +0700</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Muhammad Aminudin</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan di Gunung Bromo masih berlangsung, akses wisata ditutup hingga 15 Agustus 2026. Wisatawan dapat mengajukan refund atau reschedule tiket.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614598/karhutla-belum-padam-penutupan-bromo-diperpanjang-hingga-15-agustus</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/09/11/belum-padam-gunung-bromo-hangus-dilalap-api-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Ternyata Dedi Congor Sudah Jadi Tersangka</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:03:51 +0700</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Tim deticom</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Dedi juga terjerat kasus gratifikasi yang kasusnya diselidiki kepolisian sejak 2023.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614589/ternyata-dedi-congor-sudah-jadi-tersangka</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/08/pns-bea-cukai-ahmad-dedi-ad-lari-usai-diperiksa-kpk-demi-menghindari-wartawan-adrial-akbardetikcom-1778241473937_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Media Malaysia Soroti Asap Karhutla di Kalimantan Terbawa ke Sarawak</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:53:47 +0700</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Azhar Bagas Ramadhan</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Media Malaysia melaporkan kualitas udara memburuk akibat kabut asap dari Kalimantan. Sepuluh wilayah di Malaysia, terutama Sarawak.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614585/media-malaysia-soroti-asap-karhutla-di-kalimantan-terbawa-ke-sarawak</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/03/ratusan-titik-panas-terdeteksi-karhutla-ancam-sejumlah-wilayah-kalbar-1785728076376_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Terungkap Negara Rugi Rp 622 M saat Yaqut Didakwa Kasus Kuota Haji</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:30:55 +0700</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Tim detikcom</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Mantan Menag Yaqut Cholil Qoumas didakwa korupsi kuota haji 2023-2024, merugikan negara Rp 622 miliar. Jaksa ungkap detail kerugian dan keterlibatan pihak lain.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8614578/terungkap-negara-rugi-rp-622-m-saat-yaqut-didakwa-kasus-kuota-haji</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/eks-menag-yaqut-didakwa-perkara-kuota-haji-negara-disebut-rugi-rp622-miliar-1786428544180_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Rencana Pemerintah Batasi Pertalite buat Orang Kaya</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:30:49 +0700</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Pemerintah berencana memperketat pembelian bahan bakar minyak (BBM) Pertalite.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8614581/rencana-pemerintah-batasi-pertalite-buat-orang-kaya</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2015/07/27/a1dfc702-9caf-415e-aa20-a367dad1b9dc_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Pernak-pernik HUT RI Jadi Ladang Cuan Pedagang Musiman di Pasar Minggu</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:00:01 +0700</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Gilang Faturahman</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Menjelang HUT ke-81 RI, pedagang musiman ramai menjajakan pernak-pernik kemerdekaan. Beragam atribut merah putih dijual dengan harga bervariasi.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8614389/pernak-pernik-hut-ri-jadi-ladang-cuan-pedagang-musiman-di-pasar-minggu</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/11/pernak-pernik-hut-ri-jadi-ladang-cuan-pedagang-musiman-di-pasar-minggu-1786457391316.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Ada Aturan Baru, Driver Ojol Dijamin Tetap Dapat BHR</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:30:48 +0700</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Herdi Alif Al Hikam</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Driver ojek online (ojol) akan tetap mendapatkan bonus hari raya (BHR) Lebaran meskipun statusnya berubah jadi pengusaha mikro.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8614576/ada-aturan-baru-driver-ojol-dijamin-tetap-dapat-bhr</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/11/10/ilustrasi-driver-ojol-1762782634885_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Congrats! Cristiano Ronaldo Menikahi Georgina Setelah 10 Tahun</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:57:53 +0700</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Desi Puspasari</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Cristiano Ronaldo menikahi Georgina Rodriguez setelah 10 tahun bersama. Pernikahan berlangsung intim di Cascais, Portugal, dihadiri kelima anak mereka.</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8614587/congrats-cristiano-ronaldo-menikahi-georgina-setelah-10-tahun</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/04/13/cristiana-ronaldo-dan-georgina-rodriguez-1744546792458_169.webp?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Netanyahu Ogah Ikut Trump, Seberapa Kuat Israel Serang Iran Sendirian?</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:35:25 +0700</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Israel dilaporkan sedang mempersiapkan kemungkinan melakukan serangan sepihak ke Iran jika perang Washington vs Teheran berakhir.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260811203247-120-1391215/netanyahu-ogah-ikut-trump-seberapa-kuat-israel-serang-iran-sendirian</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/09/28/benjamin-netanyahu-1759026599434_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Malaysia Kirim Penyidik ke RI, Gali Informasi Kasus Pilot Bawa Narkoba</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:07:42 +0700</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Empat petugas Departemen Investigasi Kejahatan Narkotika Malaysia tiba di Jakarta, untuk mengusut kasus pilot yang kedapatan menyelundupkan narkoba ke RI.</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260812065631-106-1391260/malaysia-kirim-penyidik-ke-ri-gali-informasi-kasus-pilot-bawa-narkoba</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/03/14/ilustrasi-bendera-malaysia_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Trump Diam-diam Ganti Pesawat sampai Vonis Mati Bashar Al Assad</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:31:37 +0700</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Trump disebut ganti pesawat dari Air Force One ke pesawat kecil karena diancam dibunuh sampai Bashar Al Assad divonis mati.</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260812062514-134-1391255/trump-diam-diam-ganti-pesawat-sampai-vonis-mati-bashar-al-assad</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/03/22/presiden-as-donald-trump-1774175276156_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Satu WNI Dikabarkan Tewas Kena Serangan Houthi, Kemlu RI Buka Suara</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:00:42 +0700</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Kemlu RI disebut masih dalam proses verifikasi informasi soal satu ABK WNI yang dikabarkan tewas kena serangan Houthi di Yaman.</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260812055450-120-1391249/satu-wni-dikabarkan-tewas-kena-serangan-houthi-kemlu-ri-buka-suara</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2018/04/19/842fe7c6-b37b-4e52-8f34-3eb722ad1ed3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Ini Menantu Sultan Brunei yang Pernah Viral</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 05:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Menantu Sultan Brunei Darussalam Sultan Bolkiah, Robiatul Adawiyyah, menjadi sorotan usai gelar kerajaan dicopot karena tindakan yang dianggap tak senonoh.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260811190010-106-1391186/ini-menantu-sultan-brunei-yang-pernah-viral</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/01/15/akad-nikah-pangeran-abdul-mateen-dan-anisha-rosnah_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>KAI Tebar Promo Spesial 17 Agustus 2026, Tiket Kereta Diskon 17 Persen dan Tarif KRL-LRT Rp8</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:45:52 +0700</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>KAI beri promo spesial 17 Agustus 2026 berupa diskon 17 persen untuk KA Jarak Jauh kelas ekonomi komersial dan tarif Rp8 untuk KRL-LRT Jabodetabek.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7867190/kai-tebar-promo-spesial-17-agustus-2026-tiket-kereta-diskon-17-persen-dan-tarif-krl-lrt-rp8</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/l4jTIvYBS-FFEYFIp7YKBVkJAZk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Daftar-Kereta-Api-yang-Punya-Tarif-Khusus-di-Rute-Jogja-Solo.jpg</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Yogyakarta, Rabu 12 Agustus 2026, BMKG: Didominasi Cerah</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:43:30 +0700</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Berikut prakiraan cuaca di  Provinsi Yogyakarta pada Rabu (12/8/2026). Menurut BMKG, mayoritas wilayah di Yogyakarta cuacanya akan cerah.</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867189/prakiraan-cuaca-yogyakarta-rabu-12-agustus-2026-bmkg-didominasi-cerah</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/_NtT6j7i5suz6vLyHHQ1z3sEhbQ=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pemandangan-kawasan-Tugu-Pal-Putih-Yogyakarta.jpg</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Jabodetabek Rabu, 12 Agustus 2026: Jakarta, Depok, Tangerang, dan Bekasi Cerah</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:42:45 +0700</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>BMKG memprakirakan wilayah Jakarta, Depok, Tangerang, dan Bekasi akan cerah hari ini, Rabu (12/8/2026). Sementara Bogor diprediksi berawan.</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/metropolitan/7867188/prakiraan-cuaca-jabodetabek-rabu-12-agustus-2026-jakarta-depok-tangerang-dan-bekasi-cerah</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/Ew22ZWpIXWs0i0Fg5jOcsd0PKDk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-sekali.jpg</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Daftar 14 Kantor hingga Mobil di Pemkab Puncak Papua Tengah Dibakar Massa Usai Penyaluran Dana Desa</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:41:30 +0700</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Sejumlah fasilitas kantor Pemerintahan Kabupaten Puncak, Papua Tengah dibakar massa usai penyaluran Dana Desa (DD) tahap pertama reguler.</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867187/daftar-14-kantor-hingga-mobil-di-pemkab-puncak-papua-tengah-dibakar-massa-usai-penyaluran-dana-desa</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/cVdEniplHAMcwAYRxg18gGEMQhI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kolase-Pembakaran-Kantor-Pemerintahan-di-Papua-Tengah_1.jpg</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>IHSG Diperkirakan Kembali Menguat, Investor Wait And See Hasil Review MSCI</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:41:19 +0700</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>IHSG hari ini diperkirakan kembali menguat setelah melemah 97,49 poin pada perdagangan Selasa kemarin.</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/bisnis/7867186/ihsg-diperkirakan-kembali-menguat-investor-wait-and-see-hasil-review-msci</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/38xkcDnGiMqEuv_AZwgYcCu6fxg=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/dilanda-corona-ihsg-melemah_20200305_145008.jpg</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Unsur Pidana dalam Temuan 996 Senjata di Sekolah, Pengamat: Sangat Tidak Masuk Akal</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:40:15 +0700</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Temuan 996 senjata di sekolah dinilai berpotensi mengandung unsur pidana, terutama terkait izin, kepemilikan, dan penyimpanannya.</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867185/unsur-pidana-dalam-temuan-996-senjata-di-sekolah-pengamat-sangat-tidak-masuk-akal</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tFYjnCW32FN1ESklLmCo5RFVxmM=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Pengamanan-temuan-senjata-di-sekolah.jpg</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Kota Surabaya, Kediri, Madiun, Blitar, Rabu 12 Agustus 2026: Cerah Berawan</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:38:37 +0700</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Simak prakiraan cuaca di Kota Surabaya, Kediri, Madiun, dan Blitar pada Rabu (12/8/2026). Seluruh wilayah tersebut diprediksi cerah berawan.</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867184/prakiraan-cuaca-kota-surabaya-kediri-madiun-blitar-rabu-12-agustus-2026-cerah-berawan</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/d6Z05zmYE-ZlbOieHWf6t6Q66ws=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-berawan-247.jpg</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Sejarah Hari Wanita TNI Angkatan Udara atau HUT ke-63 WARA, Diperingati 12 Agustus</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:34:08 +0700</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Hari Wanita TNI Angkatan Udara atau HUT ke-63 WARA diperingati pada 12 Agustus 2026. Sejarahnya tak lepas dari peran TNI wanita tahun 1960-an.</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867183/sejarah-hari-wanita-tni-angkatan-udara-atau-hut-ke-63-wara-diperingati-12-agustus</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/PG2vUXka7u8UBvfUMgrwHGXso1Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/TNl-WANlTA-345343453.jpg</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Eks Persib Kena Gocek Milik dalam Kemenangan Juventus, Pelatih Palermo: Penting Pemain Tak Cedera</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:29:31 +0700</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Mantan pemain Persib Bandung, Federico Barba, kena gocek Arkadiusz Milik saat Palermo dikalahkan Juventus 2-0 di Australia.</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/superskor/7867182/eks-persib-kena-gocek-milik-dalam-kemenangan-juventus-pelatih-palermo-penting-pemain-tak-cedera</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/RvTZVRH7K9SPllyxhEm7y5TuadI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Penyerang-Persebaya-Surabaya-Bruno-Moreira-saat-dihadang-bek-Persib-Bandung-Federico-Barba.jpg</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>An Se-young Menuju Kejuaraan Dunia BWF 2026 dengan Membawa Misi Balas Dendam</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:18:06 +0700</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Misi balas dendam dibawa oleh An Se-young dalam perjalanannya menuju gelaran bergengsi Kejuaraan Dunia BWF 2026 di New Delhi.</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7867181/an-se-young-menuju-kejuaraan-dunia-bwf-2026-dengan-membawa-misi-balas-dendam</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/uhMannKbPjP6hOu9TqQPUB0D_F8=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Selebrasi-An-Se-young-Final-Malaysia-Open-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Komentar Ibunda Asila Maisa soal Putrinya Jadi Saksi Laporan Rizky Billar, Soroti Kebenaran</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:16:54 +0700</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Asila Maisa diperiksa sebagai saksi dalam laporan Rizky Billar soal hoaks. Sang ibunda, Avi Basalamah, ikut memberikan dukungan.</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7867180/komentar-ibunda-asila-maisa-soal-putrinya-jadi-saksi-laporan-rizky-billar-soroti-kebenaran</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/ojP31E7SsmHSHs02l0SLO4UZXrI=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Asila-Maisa.jpg</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Aripat Dituding Numpang Hidup, Nathalie Holscher Bongkar Alasan Boyong Suami Tinggal di Rumahnya</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:15:11 +0700</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Arief Fadli atau akrab disapa Aripat dituding hanya numpang hidup, Nathalie Holscher membongkar alasan mengajak sang suami tinggal di rumahnya.</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7867179/aripat-dituding-numpang-hidup-nathalie-holscher-bongkar-alasan-boyong-suami-tinggal-di-rumahnya</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/K_73CdJeZNrfun2dJLzXfN_pbdc=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Nathalie-Holscher-1-21102025.jpg</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Korut Tembakkan Rudal Balistik ke Timur Laut Korsel, di Luar ZEE Jepang</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:14:12 +0700</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Militer Korea Utara menembakkan setidaknya satu rudal balistik ke arah Laut Timur Korea Selatan pada Rabu pagi, 12 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/internasional/7867178/korut-tembakkan-rudal-balisti-ke-ke-timur-laut-korsel-di-luar-zee-jepang</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/R-5EYr5JxAhkh7uBXPpFZNkS-oU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Rudal-balistik-Korut-2025-OK.jpg</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca Bandung Raya Rabu, 12 Agustus 2026: Kota Bandung dan Cimahi Cerah</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:14:00 +0700</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Cuaca di seluruh wilayah Bandung Raya pada Rabu (12/8/2026) diprakirakan cerah, termasuk Kota Bandung dan Cimahi.</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867177/prakiraan-cuaca-bandung-raya-rabu-12-agustus-2026-kota-bandung-dan-cimahi-cerah</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/lDgUVS5zQ1sLN8t3mHbweeriZkY=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/cuaca-cerah-berawan-xx.jpg</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Jangan Pakai Nama Samaran, Ini Cara Ortu Kenalkan Organ Intim pada Anak</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:13:30 +0700</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Dokter Septian menjelaskan orang tua tidak perlu menggunakan nama samaran untuk mengenalkan organ intim kepada anak.</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/kesehatan/7867176/jangan-pakai-nama-samaran-ini-cara-ortu-kenalkan-organ-intim-pada-anak</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/5JzZqcU8Zxy0KWyxDlGXo7OMqvA=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Anak-anak-SD-Kanisius-Solo.jpg</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Keluarga Sutrimo Dijaga Ketat Jelang Pembongkaran Makam di Banyumas</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:07:08 +0700</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Kuasa Hukum Aan Rohaeni ungkap keamanan dan kondisi keluarga Sutrimo jelang pembongkaran makam atau ekshumasi di Banyumas, Rabu (12/8/2026).</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/nasional/7867175/keluarga-sutrimo-dijaga-ketat-jelang-pembongkaran-makam-di-banyumas</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/CawjQmYsx6SChqFOdefPkSh2M4U=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kematian-Sutrimo-Dilaporkan-ke-Polisi-oleh-Keluarga.jpg</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Dikecam Netizen usai Peluk Vokalis JET di Panggung, Aldi Taher Bersuara:Gue Peluk Bukan Colong Gitar</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:06:03 +0700</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Aldi Taher dikecam netizen usai memeluk vokalis band JET, Nic Cester, di atas panggung The Sounds Project.</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/seleb/7867174/dikecam-netizen-usai-peluk-vokalis-jet-di-panggung-aldi-taher-bersuarague-peluk-bukan-colong-gitar</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/I75QaFzNwI10YfC_5Suv_vcBvaU=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Aldi-taher-bisnis-ayam.jpg</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Berawal dari Penyaluran Dana Desa, 7 Kantor Pemerintah Kabupaten Puncak Papua Tengah Dibakar</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:50:30 +0700</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Pembakaran kantor diduga buntut dari penyaluran Dana Desa (DD) tahap pertama reguler, Selasa (11/8/2026).</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867173/berawal-dari-penyaluran-dana-desa-7-kantor-pemerintah-kabupaten-puncak-papua-tengah-dibakar</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/tDk7IObInGCnZb1nWhJ5FdYEj4Q=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/ilustrasi-kebakarannnnnnnnnnnnnnnnnnnn.jpg</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Gedung Biro Kesra di Kantor Gubernur Kalteng Kebakaran</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:37:03 +0700</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Berdasarkan laporan resmi dari tim kedaruratan, informasi kebakaran diterima petugas dari laporan masyarakat pada pukul 02.40 WIB.</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/regional/7867172/gedung-biro-kesra-di-kantor-gubernur-kalteng-kebakaran</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/egPXVEaAqYXtz_9JckAfbocqhvk=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Kebakaran-di-Kompleks-Kantor-Gubernur-kalteng.jpg</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Launch MotoGP 2027 Berlokasi di Rio de Janeiro, Brasil Jadi Negara Ketiga dalam 3 Tahun</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:33:48 +0700</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Redaksi Tribunnews</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>MotoGP menunjuk Rio de Janeiro, Brasil, sebagai lokasi launch musim 2027 sekaligus melanjutkan tradisi di lokasi berbeda.</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>https://www.tribunnews.com/sport/7867171/launch-motogp-2027-berlokasi-di-rio-de-janeiro-brasil-jadi-negara-ketiga-dalam-3-tahun</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>https://asset.tribunnews.com/QWRdNYbbfG5s6YXga5PrKpnEFfo=/148x99/filters:quality(30):format(webp):focal(0.5x0.5:0.5x0.5)/tribunnews/foto/bank/originals/Sprint-Race-MotoGP-Amerika-2026.jpg</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Tribunnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Bantu Petani Lebih Efisien, 13 Sprayer Pestisida Disalurkan ke Indramayu-Majalengka</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:38:12 +0700</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Satria K Yudha</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- PT Perusahaan Perdagangan Indonesia (Persero) atau PPI menyalurkan 13 unit sprayer pestisida kepada gabungan kelompok tani (Gapoktan) di Kabupaten Indramayu dan Kabupaten Majalengka, Jawa Barat. Bantuan tersebut...</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjmsfo416/bantu-petani-lebih-efisien-13-sprayer-pestisida-disalurkan-ke-indramayumajalengka</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/penyaluran-bantuan-13-unit-sprayer-pestisida-kepada-gabungan-kelompok_260812073735-603.jpeg</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Pertanian</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Pemerintah Ancam Cabut Izin Pelaku Manipulasi Harga Pakan dan Telur</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, SURABAYA -- Menteri Pertanian (Mentan) Andi Amran Sulaiman mengancam mencabut izin usaha pelaku manipulasi harga pakan dan telur guna menjaga stabilitas pasar dan melindungi peternak nasional.
+“Bagi siapa pun yang...</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjmrwi423/pemerintah-ancam-cabut-izin-pelaku-manipulasi-harga-pakan-dan-telur</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/menteri-pertanian-amran-sulaiman-mengunjungi-peternakan-ayam-_190130090143-326.jpg</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Kemenpar Dukung InJourney-Garuda Kasih Tiket Gratis untuk Wisman</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:00:48 +0700</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Gita Amanda</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA -- Kementerian Pariwisata (Kemenpar) mendukung kolaborasi InJourney dan Garuda Indonesia dalam menghadirkan program Free Domestic Flight (FDF) dengan menyediakan 170.845 kursi penerbangan bagi wisatawan mancanegara (wisman) pemegang tiket...</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjmqpc423/kemenpar-dukung-injourneygaruda-kasih-tiket-gratis-untuk-wisman</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/020424200-1684842868-830-556.jpg</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Makam Sutrimo Dibongkar Hari Ini, Polisi Cari Petunjuk Kematian Tak Wajar</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:15:34 +0700</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya menggelar ekshumasi jenazah Sutrimo di Banyumas hari ini untuk mengungkap penyebab kematiannya yang dinilai tidak wajar.</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267627/makam-sutrimo-dibongkar-hari-ini-polisi-cari-petunjuk-kematian-tak-wajar</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/Ac0CwWSgaQOzoD0dmfbEg4_UyMk=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9312458/original/059177100_1785493658-IMG_1805.jpg</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Kebakaran Melanda Pabrik Bingkai di Duren Sawit</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:15:03 +0700</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Kebakaran Pabrik Bingkai melanda sebuah pabrik di Duren Sawit, Jakarta Timur, dini hari. Sekitar 100 personel damkar masih berjibaku memadamkan api.</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267632/kebakaran-melanda-pabrik-bingkai-di-duren-sawit</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/MwKrlqCPortK2p2e5h-_z2L7AFU=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321698/original/080400300_1786493694-ilustrasi_kebakaran.jpg</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Dakwaan Jaksa vs Bantahan Eks Menag Yaqut di Sidang Korupsi Kuota Haji</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:01:41 +0700</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Dalam sidang perdana, jaksa membeberkan dugaan aliran uang dan kerugian negara Rp622 miliar, sementara Yaqut membantah menerima uang dan mempertanyakan dasar dakwaan tersebut.</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267602/dakwaan-jaksa-vs-bantahan-eks-menag-yaqut-di-sidang-korupsi-kuota-haji</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/stAlPACGZORRu5DU5poKMV3z6yU=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321159/original/065738600_1786430944-ya4.jpg</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>KH Anwar Zahid Cerita Detik-Detik Mobilnya Ditabrak Truk</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 06:51:21 +0700</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>KH Anwar Zahid menceritakan kondisi dirinya setelah mobil yang ditumpanginya ditabrak truk trailer saat mengantre di lokasi perbaikan jalan.</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267625/kh-anwar-zahid-cerita-detik-detik-mobilnya-ditabrak-truk</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/cPtrbZUIV1_7u3BqpwQw6fs1kG4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9321696/original/090135600_1786492180-kh-anwar-zahid-saat-mengisi-pengajian-di-desa-sije-20260811064255.jpg</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Pemerintah Pastikan Tak Ada Peningkatan Ancaman Jelang HUT RI</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:12:46 +0700</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Pemerintah memastikan situasi keamanan nasional terkendali menjelang HUT ke-81 RI dan meminta masyarakat waspada terhadap informasi di ruang digital.</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8267631/pemerintah-pastikan-tak-ada-peningkatan-ancaman-jelang-hut-ri</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/NIqGLJIZgyZbSe5Fg4VkaJUo6vs=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9316148/original/057906600_1785915445-0db335b9-1614-4759-aad0-edd8c8ddac02.jpg</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Kejari Kembali Sita Rp 1,24 Miliar dalam Kasus Korupsi Tunjangan Perumahan DPRD Ponorogo</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:59:19 +0700</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Kejari Ponorogo kembali menyita uang dalam penyidikan kasus dugaan korupsi tunjangan perumahan anggota DPRD Ponorogo</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/08/12/075757478/kejari-kembali-sita-rp-124-miliar-dalam-kasus-korupsi-tunjangan-perumahan</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/HF0Efvp2vYROPBvSi_cA43V2glE=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/12/6a7bbcce32d57.jpg</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Bola</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Jakarta Siapkan 2 Lapangan Latihan untuk Tunjang FIFA ASEAN Cup 2026</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:59:19 +0700</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Jakarta menyiapkan dua lapangan latihan untuk mendukung penyelenggaraan FIFA ASEAN Cup 2026.</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>https://bola.kompas.com/read/2026/08/12/07291188/jakarta-siapkan-2-lapangan-latihan-untuk-tunjang-fifa-asean-cup-2026</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/Ja9CNBTTNvY6v9XN4pb6taf8pQ8=/0x133:1600x1200/1200x675/filters:watermark(data/photo/2026/01/30/697c8163c3944.png,0,-0,1)/data/photo/2026/08/10/6a796e6e6b9f0.jpg</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Dinamika Jelang Muktamar Ke-35 NU, Muncul Usulan Ketum PBNU Ditunjuk Langsung Rais Aam</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Wed, 12 Aug 2026 07:59:19 +0700</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Dinamika jelang Muktamar NU ke-35, usulan sistem pemilihan muncul, termasuk penguatan AHWA dan sistem voting.</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/12/07021891/dinamika-jelang-muktamar-ke-35-nu-muncul-usulan-ketum-pbnu-ditunjuk-langsung</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/baEBJu0N3bXRNX-SA8cuhT74W7c=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/06/6a73e1aa9f4de.jpg</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I81"/>
+  <autoFilter ref="A1:I133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>